<commit_message>
Publish Duisburg_2019_WC, Poznan_2019_WC, Shaoxing_2019_MAR, Szeged_2019_WCH
</commit_message>
<xml_diff>
--- a/events/Shaoxing_2019_MAR/Shaoxing_2019_MAR_Results.xlsx
+++ b/events/Shaoxing_2019_MAR/Shaoxing_2019_MAR_Results.xlsx
@@ -3471,6 +3471,11 @@
           <t>00:16:42.740</t>
         </is>
       </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>47779</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5459,6 +5464,11 @@
           <t>00:15:43.180</t>
         </is>
       </c>
+      <c r="R76" t="inlineStr">
+        <is>
+          <t>148720</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -10618,6 +10628,11 @@
           <t>00:15:41.380</t>
         </is>
       </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>47779</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -25003,6 +25018,11 @@
       <c r="P366" t="inlineStr">
         <is>
           <t>02:04:34.760</t>
+        </is>
+      </c>
+      <c r="R366" t="inlineStr">
+        <is>
+          <t>47779</t>
         </is>
       </c>
     </row>
@@ -31562,7 +31582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D343"/>
+  <dimension ref="A1:D345"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -39111,6 +39131,50 @@
         </is>
       </c>
     </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>47779</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Kristina</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>BEDEC</t>
+        </is>
+      </c>
+      <c r="D344" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>148720</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Julian</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>ALGANARAS</t>
+        </is>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>